<commit_message>
Add normalization Excel assignment
</commit_message>
<xml_diff>
--- a/week-01/Ex4A_GTrends.xlsx
+++ b/week-01/Ex4A_GTrends.xlsx
@@ -10,12 +10,25 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{18616136-2EC8-4F55-902F-E0383DD30EFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{936ED990-5E8D-4712-A688-A6269A842D25}"/>
+    <workbookView xWindow="8150" yWindow="150" windowWidth="10950" windowHeight="11280" xr2:uid="{936ED990-5E8D-4712-A688-A6269A842D25}"/>
   </bookViews>
   <sheets>
     <sheet name="GTrends_milkshake_hamburger_202" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>